<commit_message>
python script and output update (E55)
</commit_message>
<xml_diff>
--- a/dataset.xlsx
+++ b/dataset.xlsx
@@ -28,9 +28,7 @@
     <sheet state="visible" name="proPreservation" sheetId="23" r:id="rId27"/>
     <sheet state="visible" name="value" sheetId="24" r:id="rId28"/>
     <sheet state="visible" name="discussion" sheetId="25" r:id="rId29"/>
-    <sheet state="visible" name="relocation" sheetId="26" r:id="rId30"/>
-    <sheet state="visible" name="replacement" sheetId="27" r:id="rId31"/>
-    <sheet state="visible" name="actionUndefined" sheetId="28" r:id="rId32"/>
+    <sheet state="visible" name="type" sheetId="26" r:id="rId30"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -40,13 +38,13 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={233f4a9f-9d11-4e7a-9ec7-03030684d7c9}</author>
-    <author>tc={6dd890ef-a126-4691-bf27-ca364a0bdea6}</author>
-    <author>tc={a2354a05-843c-4543-99bf-a0cbdc5635ee}</author>
-    <author>tc={b107b2ee-ec9f-4594-92c2-4e283d6e5e0d}</author>
+    <author>tc={0ae333d3-a967-4ded-8579-11f916797199}</author>
+    <author>tc={7fa7e4ca-dc65-43c5-8a0b-f38b034c297f}</author>
+    <author>tc={816104f0-58d8-4731-b885-a0eb23ff28b6}</author>
+    <author>tc={a2cfd5bf-fb59-4d9f-99c4-67d687bd04e1}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{233f4a9f-9d11-4e7a-9ec7-03030684d7c9}" ref="A7">
+    <comment authorId="0" xr:uid="{0ae333d3-a967-4ded-8579-11f916797199}" ref="A9">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -55,7 +53,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="1" xr:uid="{6dd890ef-a126-4691-bf27-ca364a0bdea6}" ref="A8">
+    <comment authorId="1" xr:uid="{7fa7e4ca-dc65-43c5-8a0b-f38b034c297f}" ref="A7">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -64,7 +62,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="2" xr:uid="{a2354a05-843c-4543-99bf-a0cbdc5635ee}" ref="A9">
+    <comment authorId="2" xr:uid="{816104f0-58d8-4731-b885-a0eb23ff28b6}" ref="A7">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -73,7 +71,7 @@
 </t>
       </text>
     </comment>
-    <comment authorId="3" xr:uid="{b107b2ee-ec9f-4594-92c2-4e283d6e5e0d}" ref="A7">
+    <comment authorId="3" xr:uid="{a2cfd5bf-fb59-4d9f-99c4-67d687bd04e1}" ref="A8">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -89,25 +87,25 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={b03dc1a1-9866-4796-bead-b0ec503fd671}</author>
-    <author>tc={fb7aee99-d08c-4602-82b7-abebf98cc520}</author>
+    <author>tc={85b33817-0f67-432a-aa67-d0894cca60bf}</author>
+    <author>tc={ab7af052-76ea-4c66-9255-e8b64880f155}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{b03dc1a1-9866-4796-bead-b0ec503fd671}" ref="B1">
+    <comment authorId="0" xr:uid="{85b33817-0f67-432a-aa67-d0894cca60bf}" ref="C1">
+      <text>
+        <t xml:space="preserve">[Threaded comment]
+ Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+	mettiamo sempre sia i controversial fact che la legacy che gli heritage concept
+</t>
+      </text>
+    </comment>
+    <comment authorId="1" xr:uid="{ab7af052-76ea-4c66-9255-e8b64880f155}" ref="B1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
 	inserire nei pro removal il fatto che le statue non tengono in considerazione le vittime o le azioni e che sarebbe bello venissero menzionate
-</t>
-      </text>
-    </comment>
-    <comment authorId="1" xr:uid="{fb7aee99-d08c-4602-82b7-abebf98cc520}" ref="C1">
-      <text>
-        <t xml:space="preserve">[Threaded comment]
- Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-	mettiamo sempre sia i controversial fact che la legacy che gli heritage concept
 </t>
       </text>
     </comment>
@@ -118,10 +116,10 @@
 <file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={374b2748-323a-463a-8b71-3d8dd8a4e897}</author>
+    <author>tc={b29fb5dc-bae5-4cc8-b84f-d68c703654ff}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{374b2748-323a-463a-8b71-3d8dd8a4e897}" ref="B1">
+    <comment authorId="0" xr:uid="{b29fb5dc-bae5-4cc8-b84f-d68c703654ff}" ref="B1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -135,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1623" uniqueCount="888">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1621" uniqueCount="893">
   <si>
     <t>monument_id</t>
   </si>
@@ -2969,13 +2967,13 @@
     <t>The discussion that arises from different stakeholders' perspectives on Colombo statue controversy</t>
   </si>
   <si>
-    <t>relocation_action</t>
+    <t>type_relocation</t>
   </si>
   <si>
     <t>The discussion that arises from different stakeholders' perspectives on Montanelli statue controversy</t>
   </si>
   <si>
-    <t>undefined_action</t>
+    <t>type_removal;type_keeping;type_contextualization</t>
   </si>
   <si>
     <t>The discussion that arises from different stakeholders' perspectives on Hagenbeck statue controversy</t>
@@ -2987,7 +2985,7 @@
     <t>The discussion that arises from different stakeholders' perspectives on Wollstonecraftstatue controversy</t>
   </si>
   <si>
-    <t>replacement_action</t>
+    <t>type_replacement</t>
   </si>
   <si>
     <t>The discussion that arises from different stakeholders' perspectives on Colbert statue controversy</t>
@@ -3005,7 +3003,7 @@
     <t>The discussion that arises from different stakeholders' perspectives on Savile statue controversy</t>
   </si>
   <si>
-    <t>relocation_id</t>
+    <t>type_id</t>
   </si>
   <si>
     <t>action_proposal_label</t>
@@ -3014,16 +3012,31 @@
     <t>Relocation</t>
   </si>
   <si>
-    <t>replacement_id</t>
-  </si>
-  <si>
-    <t>Replace the statue with a new one</t>
-  </si>
-  <si>
-    <t>undefined_action_id</t>
-  </si>
-  <si>
-    <t>The discussion among the stakeholders did not lead to a remedy action</t>
+    <t>Replacement of the statue with a new one</t>
+  </si>
+  <si>
+    <t>type_demolition</t>
+  </si>
+  <si>
+    <t>Demolition</t>
+  </si>
+  <si>
+    <t>type_keeping</t>
+  </si>
+  <si>
+    <t>Keeping</t>
+  </si>
+  <si>
+    <t>type_removal</t>
+  </si>
+  <si>
+    <t>Removal</t>
+  </si>
+  <si>
+    <t>type_contextualization</t>
+  </si>
+  <si>
+    <t>Contextualization</t>
   </si>
 </sst>
 </file>
@@ -3500,14 +3513,6 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
-<file path=xl/drawings/drawing27.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing28.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
@@ -3538,8 +3543,8 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="Anna Pasetto" id="{56573dd9-a98c-4f86-9cfb-8ef644742e8a}" providerId="google-sheets"/>
-  <x18tc:person displayName="Alice P" id="{a2de8c48-cca5-4d15-a5d7-395b6f355ae2}" providerId="google-sheets"/>
+  <x18tc:person displayName="Anna Pasetto" id="{3f1a5ab4-c8be-4d3b-948c-b47f5b22a4b0}" providerId="google-sheets"/>
+  <x18tc:person displayName="Alice P" id="{960e522f-40a2-47a6-8ff4-80e2dacf1f26}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -3739,16 +3744,16 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A7" dT="2026-01-09T08:51:03.00" personId="{a2de8c48-cca5-4d15-a5d7-395b6f355ae2}" id="{233f4a9f-9d11-4e7a-9ec7-03030684d7c9}" done="1">
+  <x18tc:threadedComment ref="A7" dT="2026-01-09T08:51:03.00" personId="{960e522f-40a2-47a6-8ff4-80e2dacf1f26}" id="{7fa7e4ca-dc65-43c5-8a0b-f38b034c297f}" done="1">
     <x18tc:text xml:space="preserve">Colbert</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A8" dT="2026-01-09T08:51:13.00" personId="{a2de8c48-cca5-4d15-a5d7-395b6f355ae2}" id="{6dd890ef-a126-4691-bf27-ca364a0bdea6}" done="1">
+  <x18tc:threadedComment ref="A8" dT="2026-01-09T08:51:13.00" personId="{960e522f-40a2-47a6-8ff4-80e2dacf1f26}" id="{a2cfd5bf-fb59-4d9f-99c4-67d687bd04e1}" done="1">
     <x18tc:text xml:space="preserve">Colbert</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A7" dT="2026-01-09T08:50:29.00" personId="{a2de8c48-cca5-4d15-a5d7-395b6f355ae2}" id="{b107b2ee-ec9f-4594-92c2-4e283d6e5e0d}" done="1">
+  <x18tc:threadedComment ref="A7" dT="2026-01-09T08:50:29.00" personId="{960e522f-40a2-47a6-8ff4-80e2dacf1f26}" id="{816104f0-58d8-4731-b885-a0eb23ff28b6}" done="1">
     <x18tc:text xml:space="preserve">Colbert</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="A9" dT="2026-01-09T08:51:21.00" personId="{a2de8c48-cca5-4d15-a5d7-395b6f355ae2}" id="{a2354a05-843c-4543-99bf-a0cbdc5635ee}" done="1">
+  <x18tc:threadedComment ref="A9" dT="2026-01-09T08:51:21.00" personId="{960e522f-40a2-47a6-8ff4-80e2dacf1f26}" id="{0ae333d3-a967-4ded-8579-11f916797199}" done="1">
     <x18tc:text xml:space="preserve">Colbert</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -3756,10 +3761,10 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B1" dT="2026-01-12T13:59:21.00" personId="{56573dd9-a98c-4f86-9cfb-8ef644742e8a}" id="{b03dc1a1-9866-4796-bead-b0ec503fd671}" done="1">
+  <x18tc:threadedComment ref="B1" dT="2026-01-12T13:59:21.00" personId="{3f1a5ab4-c8be-4d3b-948c-b47f5b22a4b0}" id="{ab7af052-76ea-4c66-9255-e8b64880f155}" done="1">
     <x18tc:text xml:space="preserve">inserire nei pro removal il fatto che le statue non tengono in considerazione le vittime o le azioni e che sarebbe bello venissero menzionate</x18tc:text>
   </x18tc:threadedComment>
-  <x18tc:threadedComment ref="C1" dT="2026-01-12T13:45:34.00" personId="{56573dd9-a98c-4f86-9cfb-8ef644742e8a}" id="{fb7aee99-d08c-4602-82b7-abebf98cc520}" done="1">
+  <x18tc:threadedComment ref="C1" dT="2026-01-12T13:45:34.00" personId="{3f1a5ab4-c8be-4d3b-948c-b47f5b22a4b0}" id="{85b33817-0f67-432a-aa67-d0894cca60bf}" done="1">
     <x18tc:text xml:space="preserve">mettiamo sempre sia i controversial fact che la legacy che gli heritage concept</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -3767,7 +3772,7 @@
 
 <file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="B1" dT="2026-01-12T14:20:36.00" personId="{56573dd9-a98c-4f86-9cfb-8ef644742e8a}" id="{374b2748-323a-463a-8b71-3d8dd8a4e897}" done="1">
+  <x18tc:threadedComment ref="B1" dT="2026-01-12T14:20:36.00" personId="{3f1a5ab4-c8be-4d3b-948c-b47f5b22a4b0}" id="{b29fb5dc-bae5-4cc8-b84f-d68c703654ff}" done="1">
     <x18tc:text xml:space="preserve">mettere i dati veri quando ci sono e quando non ci sono usare i nomi degli scenari</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -23342,7 +23347,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="23.88"/>
     <col customWidth="1" min="2" max="2" width="79.25"/>
-    <col customWidth="1" min="3" max="3" width="17.75"/>
+    <col customWidth="1" min="3" max="3" width="44.13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -23490,7 +23495,7 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="18.75"/>
-    <col customWidth="1" min="2" max="2" width="22.88"/>
+    <col customWidth="1" min="2" max="2" width="32.0"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -23517,84 +23522,44 @@
         <v>883</v>
       </c>
     </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="19.25"/>
-    <col customWidth="1" min="2" max="2" width="19.63"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="25" t="s">
+    <row r="4">
+      <c r="A4" s="14" t="s">
+        <v>875</v>
+      </c>
+      <c r="B4" s="14" t="s">
         <v>884</v>
       </c>
-      <c r="B1" s="52" t="s">
-        <v>882</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="52" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="s">
-        <v>875</v>
-      </c>
-      <c r="B3" s="14" t="s">
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="s">
         <v>885</v>
       </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="20.75"/>
-    <col customWidth="1" min="2" max="2" width="54.13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="25" t="s">
+      <c r="B5" s="14" t="s">
         <v>886</v>
       </c>
-      <c r="B1" s="52" t="s">
-        <v>882</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="27" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="52" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="s">
-        <v>871</v>
-      </c>
-      <c r="B3" s="14" t="s">
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="s">
         <v>887</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="s">
+        <v>889</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="s">
+        <v>891</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>